<commit_message>
[add] Added BKR option in the configuration and generated the corresponding summaries. Also removed mode Other in the mode choice table. #170
</commit_message>
<xml_diff>
--- a/inputs/model/survey/ACS_2023.xlsx
+++ b/inputs/model/survey/ACS_2023.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405332D-5D4A-4059-999C-1A645F262BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431991C4-D3A5-4969-B397-30BEA1DF90BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15255" yWindow="4185" windowWidth="14445" windowHeight="9405" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AutosCounty" sheetId="5" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>Number of Vehicles in Household</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>B08006: Sex of Workers by Means of ... - Census Bureau Table</t>
+  </si>
+  <si>
+    <t>B25044: Tenure by Vehicles Available - Census Bureau Table</t>
   </si>
 </sst>
 </file>
@@ -704,7 +707,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.7109375" customWidth="1"/>
@@ -721,7 +724,7 @@
     <col min="17" max="17" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -773,8 +776,11 @@
       <c r="Q1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R1" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -835,7 +841,7 @@
         <v>138949</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -896,7 +902,7 @@
         <v>542186</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -957,7 +963,7 @@
         <v>617488</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1018,7 +1024,7 @@
         <v>256989</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -1079,7 +1085,7 @@
         <v>138002</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C7">
         <v>13962</v>
       </c>
@@ -1122,7 +1128,7 @@
         <v>12643</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G8" s="6">
         <f>SUM(G2:G6)</f>
         <v>1033540</v>
@@ -1136,7 +1142,7 @@
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L9" s="9">
         <f>SUM(G8,L8)</f>
         <v>1693614</v>
@@ -1147,6 +1153,9 @@
       <c r="P9" s="9"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="R1" r:id="rId1" display="https://data.census.gov/table/ACSDT5Y2023.B25044?q=vehicles+available&amp;g=050XX00US53033,53035,53053,53061" xr:uid="{D9241D5D-319D-4884-BFCA-961A8E11D5E8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>